<commit_message>
Make attestation hermetically testable; fix a test that read production state
test_goal_is_not_met_before_the_caiq_is_filled used a sandbox claims file but
attest_self read the repo's real docs/ai-caiq/. The moment the real workbook was
generated the test started passing for the wrong reason — it was asserting against
production state, which is not a test. caiq_dir is now injectable and the three
attestation tests point at their own empty directories.

This landed in the same push as the failing test, which should not have happened:
the suite was run after the commit rather than before it.

221 tests, ruff clean, attest --self still exits 0.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Na2PJguodVtmmSUTVcm53n
</commit_message>
<xml_diff>
--- a/docs/ai-caiq/AI-CAIQ-stop-guessing-v1.1.0.xlsx
+++ b/docs/ai-caiq/AI-CAIQ-stop-guessing-v1.1.0.xlsx
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>`verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; The carried AI-CAIQ version is inspected on every run by parsing cell A1's JSON blob, not by trusting the sheet name, and a drifted workbook refuses regeneration; Every distributed surface — plugin, skill, slash-command and CLI — has been exercised by at least one live-run proof recorded in this toolchain's own ledger; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 10 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:20:f6901d9c28fd2f28, sg:26:fadb8b44cbf92e38, sg:37:82ae8f8f17419cab, sg:39:fbe37ba1a9e2b863, sg:46:1e975a983138ffd6, sg:4:276bdc000eb55277, sg:54:8bcbddcadf8f1734, sg:60:571f52205287dd41, sg:61:d8495b2ca3ac47d7, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>`verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; The carried AI-CAIQ version is inspected on every run by parsing cell A1's JSON blob, not by trusting the sheet name, and a drifted workbook refuses regeneration; Every distributed surface — plugin, skill, slash-command and CLI — has been exercised by at least one live-run proof recorded in this toolchain's own ledger; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 14 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:20:f6901d9c28fd2f28, sg:26:fadb8b44cbf92e38, sg:37:82ae8f8f17419cab, sg:39:fbe37ba1a9e2b863, sg:46:1e975a983138ffd6, sg:4:276bdc000eb55277, sg:54:8bcbddcadf8f1734, sg:60:571f52205287dd41, sg:61:d8495b2ca3ac47d7, sg:67:3b66f7dac01ccd60, sg:75:229d4e17d8b99c62, sg:81:86d629fb715c366a, sg:82:f7cc594a8b2b486b, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>`verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; The carried AI-CAIQ version is inspected on every run by parsing cell A1's JSON blob, not by trusting the sheet name, and a drifted workbook refuses regeneration; Every distributed surface — plugin, skill, slash-command and CLI — has been exercised by at least one live-run proof recorded in this toolchain's own ledger; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 10 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:20:f6901d9c28fd2f28, sg:26:fadb8b44cbf92e38, sg:37:82ae8f8f17419cab, sg:39:fbe37ba1a9e2b863, sg:46:1e975a983138ffd6, sg:4:276bdc000eb55277, sg:54:8bcbddcadf8f1734, sg:60:571f52205287dd41, sg:61:d8495b2ca3ac47d7, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>`verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; The carried AI-CAIQ version is inspected on every run by parsing cell A1's JSON blob, not by trusting the sheet name, and a drifted workbook refuses regeneration; Every distributed surface — plugin, skill, slash-command and CLI — has been exercised by at least one live-run proof recorded in this toolchain's own ledger; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 14 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:20:f6901d9c28fd2f28, sg:26:fadb8b44cbf92e38, sg:37:82ae8f8f17419cab, sg:39:fbe37ba1a9e2b863, sg:46:1e975a983138ffd6, sg:4:276bdc000eb55277, sg:54:8bcbddcadf8f1734, sg:60:571f52205287dd41, sg:61:d8495b2ca3ac47d7, sg:67:3b66f7dac01ccd60, sg:75:229d4e17d8b99c62, sg:81:86d629fb715c366a, sg:82:f7cc594a8b2b486b, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F4" s="18" t="n"/>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="E44" s="18" t="inlineStr">
         <is>
-          <t>A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Superseding no-noodles is byte-compatible: every payload in the corpus produces an identical (exit_code, stdout) through the dispatcher as through the standalone hooks; Every no-noodles surface keeps working after supersession — the three escape markers, the config chain, `grant_session_trust.sh`, `/no-noodle`, `/noodle-options`, and `risk_summary.py` parsing `observations.jsonl`. Proven by 8 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:23:a008c5fa1d367385, sg:27:ec2b4becd7c77e29, sg:36:330695993f562a6e, sg:49:4a65b4cd43d97bea, sg:56:1aa8e8cd7607771c, sg:57:f00a04ac3328aad2, sg:5:c95b7b06e158da45), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Superseding no-noodles is byte-compatible: every payload in the corpus produces an identical (exit_code, stdout) through the dispatcher as through the standalone hooks; Every no-noodles surface keeps working after supersession — the three escape markers, the config chain, `grant_session_trust.sh`, `/no-noodle`, `/noodle-options`, and `risk_summary.py` parsing `observations.jsonl`. Proven by 11 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:23:a008c5fa1d367385, sg:27:ec2b4becd7c77e29, sg:36:330695993f562a6e, sg:49:4a65b4cd43d97bea, sg:56:1aa8e8cd7607771c, sg:57:f00a04ac3328aad2, sg:5:c95b7b06e158da45, sg:70:cb61aa7cb8e712da, sg:77:195c3b7af795e666, sg:78:20569b15038d3d77), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F44" s="18" t="n"/>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Superseding no-noodles is byte-compatible: every payload in the corpus produces an identical (exit_code, stdout) through the dispatcher as through the standalone hooks; Every no-noodles surface keeps working after supersession — the three escape markers, the config chain, `grant_session_trust.sh`, `/no-noodle`, `/noodle-options`, and `risk_summary.py` parsing `observations.jsonl`. Proven by 8 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:23:a008c5fa1d367385, sg:27:ec2b4becd7c77e29, sg:36:330695993f562a6e, sg:49:4a65b4cd43d97bea, sg:56:1aa8e8cd7607771c, sg:57:f00a04ac3328aad2, sg:5:c95b7b06e158da45), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Superseding no-noodles is byte-compatible: every payload in the corpus produces an identical (exit_code, stdout) through the dispatcher as through the standalone hooks; Every no-noodles surface keeps working after supersession — the three escape markers, the config chain, `grant_session_trust.sh`, `/no-noodle`, `/noodle-options`, and `risk_summary.py` parsing `observations.jsonl`. Proven by 11 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:23:a008c5fa1d367385, sg:27:ec2b4becd7c77e29, sg:36:330695993f562a6e, sg:49:4a65b4cd43d97bea, sg:56:1aa8e8cd7607771c, sg:57:f00a04ac3328aad2, sg:5:c95b7b06e158da45, sg:70:cb61aa7cb8e712da, sg:77:195c3b7af795e666, sg:78:20569b15038d3d77), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F45" s="14" t="n"/>
@@ -5365,7 +5365,7 @@
       </c>
       <c r="E112" s="18" t="inlineStr">
         <is>
-          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 5 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:15:bf273856e947ee23, sg:31:e3f89cd814900706, sg:41:7a7f781b465c9908, sg:58:f4c71b0ec7276039, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 7 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:15:bf273856e947ee23, sg:31:e3f89cd814900706, sg:41:7a7f781b465c9908, sg:58:f4c71b0ec7276039, sg:62:840752dcd3002f50, sg:79:b41619813ad4e433, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F112" s="18" t="n"/>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="E113" s="14" t="inlineStr">
         <is>
-          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 5 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:15:bf273856e947ee23, sg:31:e3f89cd814900706, sg:41:7a7f781b465c9908, sg:58:f4c71b0ec7276039, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 7 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:15:bf273856e947ee23, sg:31:e3f89cd814900706, sg:41:7a7f781b465c9908, sg:58:f4c71b0ec7276039, sg:62:840752dcd3002f50, sg:79:b41619813ad4e433, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F113" s="14" t="n"/>
@@ -5930,7 +5930,7 @@
       </c>
       <c r="E130" s="18" t="inlineStr">
         <is>
-          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Accumulated session taint denies an egress that the identical call would have been allowed to make earlier in the same session, and the denial names the contributing artifacts; `steer` asks on first touch of a classified artifact and offers a recorded script delegation; it does not deny the first read; A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Under `bar` the model receives only a handle or summary, and an unsigned script is refused; The blank AI-CAIQ template is never modified. A fill leaves its digest and mtime unchanged, and an altered template refuses regeneration; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 17 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:14:0472ec5ce6c5572b, sg:15:bf273856e947ee23, sg:22:57dd6789598beda0, sg:23:a008c5fa1d367385, sg:32:62e9084ac5c23150, sg:33:26603829d8a2d99d, sg:39:fbe37ba1a9e2b863, sg:40:7881257b3bc9ab46, sg:41:7a7f781b465c9908, sg:47:b88eb327a02935ba, sg:48:18e04efd42076c3b, sg:49:4a65b4cd43d97bea, sg:50:bb2e261c780ea83b, sg:55:075d6757ad9fea62, sg:61:d8495b2ca3ac47d7, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>The ledger records data flow, not only actions: a read, a transform and a write are linked by an explicit derivation edge naming the artifacts and the script that joined them; Accumulated session taint denies an egress that the identical call would have been allowed to make earlier in the same session, and the denial names the contributing artifacts; `steer` asks on first touch of a classified artifact and offers a recorded script delegation; it does not deny the first read; A delegated script cannot touch live data until its paired test has passed, and cannot run at all if its digest changed after the test passed; Under `bar` the model receives only a handle or summary, and an unsigned script is refused; The blank AI-CAIQ template is never modified. A fill leaves its digest and mtime unchanged, and an altered template refuses regeneration; This toolchain's own AI-CAIQ was filled from proofs produced by this toolchain, as the last step, and every answer's evidence resolves to a verified ledger record. Proven by 24 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:12:3fd44ffa4a757a26, sg:14:0472ec5ce6c5572b, sg:15:bf273856e947ee23, sg:22:57dd6789598beda0, sg:23:a008c5fa1d367385, sg:32:62e9084ac5c23150, sg:33:26603829d8a2d99d, sg:39:fbe37ba1a9e2b863, sg:40:7881257b3bc9ab46, sg:41:7a7f781b465c9908, sg:47:b88eb327a02935ba, sg:48:18e04efd42076c3b, sg:49:4a65b4cd43d97bea, sg:50:bb2e261c780ea83b, sg:55:075d6757ad9fea62, sg:61:d8495b2ca3ac47d7, sg:62:840752dcd3002f50, sg:68:ec8a054e28749618, sg:69:96cd89574676b8cc, sg:70:cb61aa7cb8e712da, sg:71:6493aa04c046d505, sg:76:298fd8e47c3f66a8, sg:82:f7cc594a8b2b486b, sg:9:8e229db09d9d3bb6), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F130" s="18" t="n"/>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="E203" s="14" t="inlineStr">
         <is>
-          <t>Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 2 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:31:e3f89cd814900706, sg:58:f4c71b0ec7276039), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 3 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:31:e3f89cd814900706, sg:58:f4c71b0ec7276039, sg:79:b41619813ad4e433), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F203" s="14" t="n"/>
@@ -8223,7 +8223,7 @@
       </c>
       <c r="E204" s="18" t="inlineStr">
         <is>
-          <t>Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 2 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:31:e3f89cd814900706, sg:58:f4c71b0ec7276039), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>Offline by default: no runtime path performs an external network call unless anchoring is explicitly enabled, and enabling it announces itself. Proven by 3 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:31:e3f89cd814900706, sg:58:f4c71b0ec7276039, sg:79:b41619813ad4e433), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F204" s="18" t="n"/>
@@ -8669,7 +8669,7 @@
       </c>
       <c r="E219" s="14" t="inlineStr">
         <is>
-          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; A record missing the `alterations` key is refused at write, while `alterations: []` is accepted — an empty list asserts nothing was altered, a missing key means nobody looked; `verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 13 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:19:b8eed958f59d640e, sg:20:f6901d9c28fd2f28, sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:42:329f422d795cf67d, sg:45:885d91082f72292f, sg:46:1e975a983138ffd6, sg:53:1c2c321ec1d637f7, sg:6:610ab1d78e9b6ffe, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; A record missing the `alterations` key is refused at write, while `alterations: []` is accepted — an empty list asserts nothing was altered, a missing key means nobody looked; `verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 17 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:19:b8eed958f59d640e, sg:20:f6901d9c28fd2f28, sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:42:329f422d795cf67d, sg:45:885d91082f72292f, sg:46:1e975a983138ffd6, sg:53:1c2c321ec1d637f7, sg:63:9c080b5b0f116776, sg:66:901b7c2facbb70d7, sg:67:3b66f7dac01ccd60, sg:6:610ab1d78e9b6ffe, sg:74:9ea2a20a2cf96f5e, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F219" s="14" t="n"/>
@@ -8717,7 +8717,7 @@
       </c>
       <c r="E220" s="18" t="inlineStr">
         <is>
-          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; A record missing the `alterations` key is refused at write, while `alterations: []` is accepted — an empty list asserts nothing was altered, a missing key means nobody looked; `verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 13 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:19:b8eed958f59d640e, sg:20:f6901d9c28fd2f28, sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:42:329f422d795cf67d, sg:45:885d91082f72292f, sg:46:1e975a983138ffd6, sg:53:1c2c321ec1d637f7, sg:6:610ab1d78e9b6ffe, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; A record missing the `alterations` key is refused at write, while `alterations: []` is accepted — an empty list asserts nothing was altered, a missing key means nobody looked; `verify --sufficiency` reports `incomplete` and names the unpopulated evidence regime rather than claiming sufficiency it cannot back; Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 17 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:19:b8eed958f59d640e, sg:20:f6901d9c28fd2f28, sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:42:329f422d795cf67d, sg:45:885d91082f72292f, sg:46:1e975a983138ffd6, sg:53:1c2c321ec1d637f7, sg:63:9c080b5b0f116776, sg:66:901b7c2facbb70d7, sg:67:3b66f7dac01ccd60, sg:6:610ab1d78e9b6ffe, sg:74:9ea2a20a2cf96f5e, sg:8:9551f0c4ea887cb2), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F220" s="18" t="n"/>
@@ -8990,7 +8990,7 @@
       </c>
       <c r="E229" s="14" t="inlineStr">
         <is>
-          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; The sink refuses to append onto a broken or truncated chain, rather than burying the break under new entries; Sealing archives a segment and chains the next segment to the sealed digest; no ledger rotation ever truncates history; The recorder is not reachable by the agent it records: PATH-shadowing the CLI, direct ledger writes, hook-script substitution and daemon kill are each refused or detected; The blank AI-CAIQ template is never modified. A fill leaves its digest and mtime unchanged, and an altered template refuses regeneration; A full uninstall removes hooks and registrations while preserving the accumulated ledger and observation log. Proven by 15 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:17:abd9cb98a7931aac, sg:18:0a53a808e1826a22, sg:1:2da04769bddc3d6b, sg:28:3d79c978f5f94865, sg:2:3a6ad16a3f7b631b, sg:33:26603829d8a2d99d, sg:35:a32f87f5a73d99c7, sg:42:329f422d795cf67d, sg:43:f2f5bee2bc12f523, sg:44:5524171aae0946b5, sg:52:2e7f22f8c6c1a019, sg:55:075d6757ad9fea62, sg:59:d3094004aa13722e), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>A keyed chain defeats truncate-and-recompute. Without the session key held in the OS keychain, a forged chain that is internally consistent still fails verification; The sink refuses to append onto a broken or truncated chain, rather than burying the break under new entries; Sealing archives a segment and chains the next segment to the sealed digest; no ledger rotation ever truncates history; The recorder is not reachable by the agent it records: PATH-shadowing the CLI, direct ledger writes, hook-script substitution and daemon kill are each refused or detected; The blank AI-CAIQ template is never modified. A fill leaves its digest and mtime unchanged, and an altered template refuses regeneration; A full uninstall removes hooks and registrations while preserving the accumulated ledger and observation log. Proven by 21 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:0:0407b42c97ccb566, sg:16:e56ac532d76e2b76, sg:17:abd9cb98a7931aac, sg:18:0a53a808e1826a22, sg:1:2da04769bddc3d6b, sg:28:3d79c978f5f94865, sg:2:3a6ad16a3f7b631b, sg:33:26603829d8a2d99d, sg:35:a32f87f5a73d99c7, sg:42:329f422d795cf67d, sg:43:f2f5bee2bc12f523, sg:44:5524171aae0946b5, sg:52:2e7f22f8c6c1a019, sg:55:075d6757ad9fea62, sg:59:d3094004aa13722e, sg:63:9c080b5b0f116776, sg:64:a3b27f1c9b025094, sg:65:ce198ee91ed4866c, sg:73:32e817ccb1c5e3ff, sg:76:298fd8e47c3f66a8, sg:80:3a06820ff0a3b2dc), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F229" s="14" t="n"/>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="E255" s="14" t="inlineStr">
         <is>
-          <t>Under `bar` the model receives only a handle or summary, and an unsigned script is refused. Proven by 2 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:32:62e9084ac5c23150, sg:50:bb2e261c780ea83b), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>Under `bar` the model receives only a handle or summary, and an unsigned script is refused. Proven by 3 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:32:62e9084ac5c23150, sg:50:bb2e261c780ea83b, sg:71:6493aa04c046d505), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F255" s="14" t="n"/>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="E256" s="18" t="inlineStr">
         <is>
-          <t>Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 4 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:53:1c2c321ec1d637f7), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 5 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:53:1c2c321ec1d637f7, sg:74:9ea2a20a2cf96f5e), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F256" s="18" t="n"/>
@@ -9858,7 +9858,7 @@
       </c>
       <c r="E257" s="14" t="inlineStr">
         <is>
-          <t>Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 4 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:53:1c2c321ec1d637f7), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
+          <t>Execution claims made by the agent are reconciled against the hook-side dispatch ledger; a fabricated or replayed claim is detected and escalated to a human. Proven by 5 record(s) in this toolchain's own keyed chain-of-custody ledger (sg:25:6dffdc5026b552d8, sg:29:6031e40cffa97197, sg:3:52bf36fd30c28c8e, sg:53:1c2c321ec1d637f7, sg:74:9ea2a20a2cf96f5e), each produced by an executable procedure and re-verified by `stop-guessing claims check`.</t>
         </is>
       </c>
       <c r="F257" s="14" t="n"/>

</xml_diff>